<commit_message>
Add tyre inspections, tread percentages, reports and remolding vendors
</commit_message>
<xml_diff>
--- a/downloads/TyreSaathi-vehicle-template.xlsx
+++ b/downloads/TyreSaathi-vehicle-template.xlsx
@@ -27,6 +27,12 @@
   <si>
     <t>Has Spare</t>
   </si>
+  <si>
+    <t>Vehicle Type (BS3/BS4/BS6)</t>
+  </si>
+  <si>
+    <t>Driver Name</t>
+  </si>
 </sst>
 </file>
 
@@ -54,7 +60,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF173F35"/>
+        <fgColor rgb="FFBD1018"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -82,6 +88,8 @@
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -97,6 +105,12 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>